<commit_message>
Update index: 16904 → 16907 [scan complete]
Scanned 3 addresses: נבון 14, נבון 15, נבון 16 (ירושלים)
Businesses found: 0
Token budget (30,000) reached — stopping scan
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:26-08-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:26-08-2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="נכסים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ממצאים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,16 +26,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
-      <color rgb="000563C1"/>
-      <u val="single"/>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00444444"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,12 +47,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00366092"/>
-        <bgColor rgb="00366092"/>
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -57,20 +64,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="001F4E79"/>
+      </left>
+      <right style="thin">
+        <color rgb="001F4E79"/>
+      </right>
+      <top style="thin">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001F4E79"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -440,14 +458,14 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -492,45 +510,17 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>עו"ד מימון ברק</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>יצחק אולשן 7, ירושלים</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>רמות</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>עורכי דין</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80213677/9010110</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>https://easy.co.il/page/26003538</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
+          <t>סריקה מיום 26-08-2026 | אינדקס התחלה: 16904 | אינדקס סיום: 16907 | כתובות נסרקו: 3 (נבון 14, נבון 15, נבון 16) | עסקים נמצאו: 0 | הערה: מגבלת טוקנים (30,000) הושגה</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>